<commit_message>
refactor(analytics): add validation outputs, fix data tables
- Add .vscode/ directory to project gitignore
- Add new CSV output files for WRS log validation and tryout metadata
- Standardize `here::here()` usage across all R scripts, replace bare here() calls
- Add jsonlite dependency and first_non_missing helper function
- Add automatic cleanup of old generated analysis files in run_all.R
- Fix column structures and add missing fields (like unanswered_count) across all output CSV tables
- Improve paired comparison analysis logic with better type casting and error handling
- Update summary report with new metadata, validation metrics, and corrected timestamps
</commit_message>
<xml_diff>
--- a/analytics/output/tables/hasil_statistik_deskriptif.xlsx
+++ b/analytics/output/tables/hasil_statistik_deskriptif.xlsx
@@ -15,6 +15,9 @@
     <sheet name="Akurasi_Bobot" sheetId="6" r:id="rId6"/>
     <sheet name="Berdasarkan_Nomor" sheetId="7" r:id="rId7"/>
     <sheet name="Transisi_Level" sheetId="8" r:id="rId8"/>
+    <sheet name="Kuesioner_Item" sheetId="9" r:id="rId9"/>
+    <sheet name="Kuesioner_Ringkasan" sheetId="10" r:id="rId10"/>
+    <sheet name="Kuesioner_Reliabilitas" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -537,96 +540,215 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P68"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>student_key</t>
+          <t>respondent_type</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>student_id</t>
+          <t>total_respondents</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>student_name</t>
+          <t>total_items</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>attempt_number</t>
+          <t>overall_mean</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>initial_level</t>
+          <t>overall_sd</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>final_level</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>total_questions</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>correct_count</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>wrong_count</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>unanswered_count</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>total_weight</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>weighted_correct</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>accuracy_percent</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>score_100</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>weighted_score_100</t>
+          <t>interpretation</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>siswa</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>34</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>4.586764705882353</v>
+      </c>
+      <c r="E2">
+        <v>0.6722797500858286</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>respondent_type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>total_respondents</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>total_items_used</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>cronbach_alpha</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>siswa</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>34</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>0.9276973769260791</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q68"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>student_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>student_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>student_name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>attempt_number</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>initial_level</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>final_level</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>total_questions</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>correct_count</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>wrong_count</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>unanswered_count</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>total_weight</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>weighted_correct</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>expected_questions</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>accuracy_percent</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>score_100</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>weighted_score_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>cms5hzr64000104l866r5zbw0</t>
         </is>
       </c>
@@ -671,16 +793,19 @@
       <c r="L2">
         <v>69</v>
       </c>
-      <c r="M2" t="b">
-        <v>1</v>
-      </c>
-      <c r="N2">
-        <v>86.66666666666667</v>
+      <c r="M2">
+        <v>15</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
       </c>
       <c r="O2">
         <v>86.66666666666667</v>
       </c>
       <c r="P2">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q2">
         <v>89.6103896103896</v>
       </c>
     </row>
@@ -731,11 +856,11 @@
       <c r="L3">
         <v>75</v>
       </c>
-      <c r="M3" t="b">
-        <v>1</v>
-      </c>
-      <c r="N3">
-        <v>100</v>
+      <c r="M3">
+        <v>15</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
       </c>
       <c r="O3">
         <v>100</v>
@@ -743,6 +868,9 @@
       <c r="P3">
         <v>100</v>
       </c>
+      <c r="Q3">
+        <v>100</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -791,11 +919,11 @@
       <c r="L4">
         <v>65</v>
       </c>
-      <c r="M4" t="b">
-        <v>1</v>
-      </c>
-      <c r="N4">
-        <v>86.66666666666667</v>
+      <c r="M4">
+        <v>15</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
       </c>
       <c r="O4">
         <v>86.66666666666667</v>
@@ -803,6 +931,9 @@
       <c r="P4">
         <v>86.66666666666667</v>
       </c>
+      <c r="Q4">
+        <v>86.66666666666667</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -851,16 +982,19 @@
       <c r="L5">
         <v>66</v>
       </c>
-      <c r="M5" t="b">
-        <v>1</v>
-      </c>
-      <c r="N5">
-        <v>93.33333333333333</v>
+      <c r="M5">
+        <v>15</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
       </c>
       <c r="O5">
         <v>93.33333333333333</v>
       </c>
       <c r="P5">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q5">
         <v>95.65217391304348</v>
       </c>
     </row>
@@ -911,16 +1045,19 @@
       <c r="L6">
         <v>78</v>
       </c>
-      <c r="M6" t="b">
-        <v>1</v>
-      </c>
-      <c r="N6">
-        <v>93.33333333333333</v>
+      <c r="M6">
+        <v>15</v>
+      </c>
+      <c r="N6" t="b">
+        <v>1</v>
       </c>
       <c r="O6">
         <v>93.33333333333333</v>
       </c>
       <c r="P6">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q6">
         <v>98.73417721518987</v>
       </c>
     </row>
@@ -971,16 +1108,19 @@
       <c r="L7">
         <v>66</v>
       </c>
-      <c r="M7" t="b">
-        <v>1</v>
-      </c>
-      <c r="N7">
-        <v>93.33333333333333</v>
+      <c r="M7">
+        <v>15</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
       </c>
       <c r="O7">
         <v>93.33333333333333</v>
       </c>
       <c r="P7">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q7">
         <v>95.65217391304348</v>
       </c>
     </row>
@@ -1031,11 +1171,11 @@
       <c r="L8">
         <v>73</v>
       </c>
-      <c r="M8" t="b">
-        <v>1</v>
-      </c>
-      <c r="N8">
-        <v>100</v>
+      <c r="M8">
+        <v>15</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
       </c>
       <c r="O8">
         <v>100</v>
@@ -1043,6 +1183,9 @@
       <c r="P8">
         <v>100</v>
       </c>
+      <c r="Q8">
+        <v>100</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1091,11 +1234,11 @@
       <c r="L9">
         <v>71</v>
       </c>
-      <c r="M9" t="b">
-        <v>1</v>
-      </c>
-      <c r="N9">
-        <v>100</v>
+      <c r="M9">
+        <v>15</v>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
       </c>
       <c r="O9">
         <v>100</v>
@@ -1103,6 +1246,9 @@
       <c r="P9">
         <v>100</v>
       </c>
+      <c r="Q9">
+        <v>100</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1151,16 +1297,19 @@
       <c r="L10">
         <v>59</v>
       </c>
-      <c r="M10" t="b">
-        <v>1</v>
-      </c>
-      <c r="N10">
-        <v>73.33333333333333</v>
+      <c r="M10">
+        <v>15</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
       </c>
       <c r="O10">
         <v>73.33333333333333</v>
       </c>
       <c r="P10">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q10">
         <v>74.68354430379746</v>
       </c>
     </row>
@@ -1211,16 +1360,19 @@
       <c r="L11">
         <v>70</v>
       </c>
-      <c r="M11" t="b">
-        <v>1</v>
-      </c>
-      <c r="N11">
-        <v>80</v>
+      <c r="M11">
+        <v>15</v>
+      </c>
+      <c r="N11" t="b">
+        <v>1</v>
       </c>
       <c r="O11">
         <v>80</v>
       </c>
       <c r="P11">
+        <v>80</v>
+      </c>
+      <c r="Q11">
         <v>82.35294117647058</v>
       </c>
     </row>
@@ -1271,16 +1423,19 @@
       <c r="L12">
         <v>63</v>
       </c>
-      <c r="M12" t="b">
-        <v>1</v>
-      </c>
-      <c r="N12">
-        <v>86.66666666666667</v>
+      <c r="M12">
+        <v>15</v>
+      </c>
+      <c r="N12" t="b">
+        <v>1</v>
       </c>
       <c r="O12">
         <v>86.66666666666667</v>
       </c>
       <c r="P12">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q12">
         <v>94.02985074626866</v>
       </c>
     </row>
@@ -1331,16 +1486,19 @@
       <c r="L13">
         <v>17</v>
       </c>
-      <c r="M13" t="b">
-        <v>1</v>
-      </c>
-      <c r="N13">
-        <v>33.33333333333333</v>
+      <c r="M13">
+        <v>15</v>
+      </c>
+      <c r="N13" t="b">
+        <v>1</v>
       </c>
       <c r="O13">
         <v>33.33333333333333</v>
       </c>
       <c r="P13">
+        <v>33.33333333333333</v>
+      </c>
+      <c r="Q13">
         <v>22.66666666666666</v>
       </c>
     </row>
@@ -1391,16 +1549,19 @@
       <c r="L14">
         <v>72</v>
       </c>
-      <c r="M14" t="b">
-        <v>1</v>
-      </c>
-      <c r="N14">
-        <v>93.33333333333333</v>
+      <c r="M14">
+        <v>15</v>
+      </c>
+      <c r="N14" t="b">
+        <v>1</v>
       </c>
       <c r="O14">
         <v>93.33333333333333</v>
       </c>
       <c r="P14">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q14">
         <v>98.63013698630137</v>
       </c>
     </row>
@@ -1451,11 +1612,11 @@
       <c r="L15">
         <v>71</v>
       </c>
-      <c r="M15" t="b">
-        <v>1</v>
-      </c>
-      <c r="N15">
-        <v>100</v>
+      <c r="M15">
+        <v>15</v>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
       </c>
       <c r="O15">
         <v>100</v>
@@ -1463,6 +1624,9 @@
       <c r="P15">
         <v>100</v>
       </c>
+      <c r="Q15">
+        <v>100</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1511,16 +1675,19 @@
       <c r="L16">
         <v>56</v>
       </c>
-      <c r="M16" t="b">
-        <v>1</v>
-      </c>
-      <c r="N16">
-        <v>80</v>
+      <c r="M16">
+        <v>15</v>
+      </c>
+      <c r="N16" t="b">
+        <v>1</v>
       </c>
       <c r="O16">
         <v>80</v>
       </c>
       <c r="P16">
+        <v>80</v>
+      </c>
+      <c r="Q16">
         <v>78.87323943661971</v>
       </c>
     </row>
@@ -1571,16 +1738,19 @@
       <c r="L17">
         <v>65</v>
       </c>
-      <c r="M17" t="b">
-        <v>1</v>
-      </c>
-      <c r="N17">
-        <v>86.66666666666667</v>
+      <c r="M17">
+        <v>15</v>
+      </c>
+      <c r="N17" t="b">
+        <v>1</v>
       </c>
       <c r="O17">
         <v>86.66666666666667</v>
       </c>
       <c r="P17">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q17">
         <v>89.04109589041096</v>
       </c>
     </row>
@@ -1631,16 +1801,19 @@
       <c r="L18">
         <v>74</v>
       </c>
-      <c r="M18" t="b">
-        <v>1</v>
-      </c>
-      <c r="N18">
-        <v>93.33333333333333</v>
+      <c r="M18">
+        <v>15</v>
+      </c>
+      <c r="N18" t="b">
+        <v>1</v>
       </c>
       <c r="O18">
         <v>93.33333333333333</v>
       </c>
       <c r="P18">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q18">
         <v>96.1038961038961</v>
       </c>
     </row>
@@ -1691,11 +1864,11 @@
       <c r="L19">
         <v>81</v>
       </c>
-      <c r="M19" t="b">
-        <v>1</v>
-      </c>
-      <c r="N19">
-        <v>100</v>
+      <c r="M19">
+        <v>15</v>
+      </c>
+      <c r="N19" t="b">
+        <v>1</v>
       </c>
       <c r="O19">
         <v>100</v>
@@ -1703,6 +1876,9 @@
       <c r="P19">
         <v>100</v>
       </c>
+      <c r="Q19">
+        <v>100</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1751,16 +1927,19 @@
       <c r="L20">
         <v>53</v>
       </c>
-      <c r="M20" t="b">
-        <v>1</v>
-      </c>
-      <c r="N20">
-        <v>73.33333333333333</v>
+      <c r="M20">
+        <v>15</v>
+      </c>
+      <c r="N20" t="b">
+        <v>1</v>
       </c>
       <c r="O20">
         <v>73.33333333333333</v>
       </c>
       <c r="P20">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q20">
         <v>70.66666666666667</v>
       </c>
     </row>
@@ -1811,16 +1990,19 @@
       <c r="L21">
         <v>62</v>
       </c>
-      <c r="M21" t="b">
-        <v>1</v>
-      </c>
-      <c r="N21">
-        <v>80</v>
+      <c r="M21">
+        <v>15</v>
+      </c>
+      <c r="N21" t="b">
+        <v>1</v>
       </c>
       <c r="O21">
         <v>80</v>
       </c>
       <c r="P21">
+        <v>80</v>
+      </c>
+      <c r="Q21">
         <v>82.66666666666667</v>
       </c>
     </row>
@@ -1871,11 +2053,11 @@
       <c r="L22">
         <v>81</v>
       </c>
-      <c r="M22" t="b">
-        <v>1</v>
-      </c>
-      <c r="N22">
-        <v>100</v>
+      <c r="M22">
+        <v>15</v>
+      </c>
+      <c r="N22" t="b">
+        <v>1</v>
       </c>
       <c r="O22">
         <v>100</v>
@@ -1883,6 +2065,9 @@
       <c r="P22">
         <v>100</v>
       </c>
+      <c r="Q22">
+        <v>100</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1931,11 +2116,11 @@
       <c r="L23">
         <v>67</v>
       </c>
-      <c r="M23" t="b">
-        <v>1</v>
-      </c>
-      <c r="N23">
-        <v>100</v>
+      <c r="M23">
+        <v>15</v>
+      </c>
+      <c r="N23" t="b">
+        <v>1</v>
       </c>
       <c r="O23">
         <v>100</v>
@@ -1943,6 +2128,9 @@
       <c r="P23">
         <v>100</v>
       </c>
+      <c r="Q23">
+        <v>100</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1991,16 +2179,19 @@
       <c r="L24">
         <v>56</v>
       </c>
-      <c r="M24" t="b">
-        <v>1</v>
-      </c>
-      <c r="N24">
-        <v>80</v>
+      <c r="M24">
+        <v>15</v>
+      </c>
+      <c r="N24" t="b">
+        <v>1</v>
       </c>
       <c r="O24">
         <v>80</v>
       </c>
       <c r="P24">
+        <v>80</v>
+      </c>
+      <c r="Q24">
         <v>83.5820895522388</v>
       </c>
     </row>
@@ -2051,16 +2242,19 @@
       <c r="L25">
         <v>76</v>
       </c>
-      <c r="M25" t="b">
-        <v>1</v>
-      </c>
-      <c r="N25">
-        <v>93.33333333333333</v>
+      <c r="M25">
+        <v>15</v>
+      </c>
+      <c r="N25" t="b">
+        <v>1</v>
       </c>
       <c r="O25">
         <v>93.33333333333333</v>
       </c>
       <c r="P25">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q25">
         <v>93.82716049382715</v>
       </c>
     </row>
@@ -2111,16 +2305,19 @@
       <c r="L26">
         <v>43</v>
       </c>
-      <c r="M26" t="b">
-        <v>1</v>
-      </c>
-      <c r="N26">
-        <v>60</v>
+      <c r="M26">
+        <v>15</v>
+      </c>
+      <c r="N26" t="b">
+        <v>1</v>
       </c>
       <c r="O26">
         <v>60</v>
       </c>
       <c r="P26">
+        <v>60</v>
+      </c>
+      <c r="Q26">
         <v>60.56338028169014</v>
       </c>
     </row>
@@ -2171,11 +2368,11 @@
       <c r="L27">
         <v>52</v>
       </c>
-      <c r="M27" t="b">
-        <v>1</v>
-      </c>
-      <c r="N27">
-        <v>80</v>
+      <c r="M27">
+        <v>15</v>
+      </c>
+      <c r="N27" t="b">
+        <v>1</v>
       </c>
       <c r="O27">
         <v>80</v>
@@ -2183,6 +2380,9 @@
       <c r="P27">
         <v>80</v>
       </c>
+      <c r="Q27">
+        <v>80</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2231,16 +2431,19 @@
       <c r="L28">
         <v>70</v>
       </c>
-      <c r="M28" t="b">
-        <v>1</v>
-      </c>
-      <c r="N28">
-        <v>93.33333333333333</v>
+      <c r="M28">
+        <v>15</v>
+      </c>
+      <c r="N28" t="b">
+        <v>1</v>
       </c>
       <c r="O28">
         <v>93.33333333333333</v>
       </c>
       <c r="P28">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q28">
         <v>90.90909090909091</v>
       </c>
     </row>
@@ -2291,16 +2494,19 @@
       <c r="L29">
         <v>57</v>
       </c>
-      <c r="M29" t="b">
-        <v>1</v>
-      </c>
-      <c r="N29">
-        <v>73.33333333333333</v>
+      <c r="M29">
+        <v>15</v>
+      </c>
+      <c r="N29" t="b">
+        <v>1</v>
       </c>
       <c r="O29">
         <v>73.33333333333333</v>
       </c>
       <c r="P29">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q29">
         <v>76</v>
       </c>
     </row>
@@ -2351,16 +2557,19 @@
       <c r="L30">
         <v>72</v>
       </c>
-      <c r="M30" t="b">
-        <v>1</v>
-      </c>
-      <c r="N30">
-        <v>93.33333333333333</v>
+      <c r="M30">
+        <v>15</v>
+      </c>
+      <c r="N30" t="b">
+        <v>1</v>
       </c>
       <c r="O30">
         <v>93.33333333333333</v>
       </c>
       <c r="P30">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q30">
         <v>93.5064935064935</v>
       </c>
     </row>
@@ -2411,16 +2620,19 @@
       <c r="L31">
         <v>74</v>
       </c>
-      <c r="M31" t="b">
-        <v>1</v>
-      </c>
-      <c r="N31">
-        <v>93.33333333333333</v>
+      <c r="M31">
+        <v>15</v>
+      </c>
+      <c r="N31" t="b">
+        <v>1</v>
       </c>
       <c r="O31">
         <v>93.33333333333333</v>
       </c>
       <c r="P31">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q31">
         <v>93.67088607594937</v>
       </c>
     </row>
@@ -2471,16 +2683,19 @@
       <c r="L32">
         <v>74</v>
       </c>
-      <c r="M32" t="b">
-        <v>1</v>
-      </c>
-      <c r="N32">
-        <v>93.33333333333333</v>
+      <c r="M32">
+        <v>15</v>
+      </c>
+      <c r="N32" t="b">
+        <v>1</v>
       </c>
       <c r="O32">
         <v>93.33333333333333</v>
       </c>
       <c r="P32">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q32">
         <v>96.1038961038961</v>
       </c>
     </row>
@@ -2531,16 +2746,19 @@
       <c r="L33">
         <v>74</v>
       </c>
-      <c r="M33" t="b">
-        <v>1</v>
-      </c>
-      <c r="N33">
-        <v>93.33333333333333</v>
+      <c r="M33">
+        <v>15</v>
+      </c>
+      <c r="N33" t="b">
+        <v>1</v>
       </c>
       <c r="O33">
         <v>93.33333333333333</v>
       </c>
       <c r="P33">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q33">
         <v>96.1038961038961</v>
       </c>
     </row>
@@ -2591,16 +2809,19 @@
       <c r="L34">
         <v>67</v>
       </c>
-      <c r="M34" t="b">
-        <v>1</v>
-      </c>
-      <c r="N34">
-        <v>86.66666666666667</v>
+      <c r="M34">
+        <v>15</v>
+      </c>
+      <c r="N34" t="b">
+        <v>1</v>
       </c>
       <c r="O34">
         <v>86.66666666666667</v>
       </c>
       <c r="P34">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q34">
         <v>91.78082191780823</v>
       </c>
     </row>
@@ -2651,16 +2872,19 @@
       <c r="L35">
         <v>71</v>
       </c>
-      <c r="M35" t="b">
-        <v>1</v>
-      </c>
-      <c r="N35">
-        <v>86.66666666666667</v>
+      <c r="M35">
+        <v>15</v>
+      </c>
+      <c r="N35" t="b">
+        <v>1</v>
       </c>
       <c r="O35">
         <v>86.66666666666667</v>
       </c>
       <c r="P35">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q35">
         <v>92.20779220779221</v>
       </c>
     </row>
@@ -2711,16 +2935,19 @@
       <c r="L36">
         <v>38</v>
       </c>
-      <c r="M36" t="b">
-        <v>1</v>
-      </c>
-      <c r="N36">
-        <v>40</v>
+      <c r="M36">
+        <v>15</v>
+      </c>
+      <c r="N36" t="b">
+        <v>1</v>
       </c>
       <c r="O36">
         <v>40</v>
       </c>
       <c r="P36">
+        <v>40</v>
+      </c>
+      <c r="Q36">
         <v>48.10126582278481</v>
       </c>
     </row>
@@ -2771,16 +2998,19 @@
       <c r="L37">
         <v>53</v>
       </c>
-      <c r="M37" t="b">
-        <v>1</v>
-      </c>
-      <c r="N37">
-        <v>73.33333333333333</v>
+      <c r="M37">
+        <v>15</v>
+      </c>
+      <c r="N37" t="b">
+        <v>1</v>
       </c>
       <c r="O37">
         <v>73.33333333333333</v>
       </c>
       <c r="P37">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q37">
         <v>70.66666666666667</v>
       </c>
     </row>
@@ -2831,16 +3061,19 @@
       <c r="L38">
         <v>48</v>
       </c>
-      <c r="M38" t="b">
-        <v>1</v>
-      </c>
-      <c r="N38">
-        <v>80</v>
+      <c r="M38">
+        <v>15</v>
+      </c>
+      <c r="N38" t="b">
+        <v>1</v>
       </c>
       <c r="O38">
         <v>80</v>
       </c>
       <c r="P38">
+        <v>80</v>
+      </c>
+      <c r="Q38">
         <v>76.19047619047619</v>
       </c>
     </row>
@@ -2891,16 +3124,19 @@
       <c r="L39">
         <v>69</v>
       </c>
-      <c r="M39" t="b">
-        <v>1</v>
-      </c>
-      <c r="N39">
-        <v>86.66666666666667</v>
+      <c r="M39">
+        <v>15</v>
+      </c>
+      <c r="N39" t="b">
+        <v>1</v>
       </c>
       <c r="O39">
         <v>86.66666666666667</v>
       </c>
       <c r="P39">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q39">
         <v>94.52054794520548</v>
       </c>
     </row>
@@ -2951,16 +3187,19 @@
       <c r="L40">
         <v>63</v>
       </c>
-      <c r="M40" t="b">
-        <v>1</v>
-      </c>
-      <c r="N40">
-        <v>86.66666666666667</v>
+      <c r="M40">
+        <v>15</v>
+      </c>
+      <c r="N40" t="b">
+        <v>1</v>
       </c>
       <c r="O40">
         <v>86.66666666666667</v>
       </c>
       <c r="P40">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q40">
         <v>84</v>
       </c>
     </row>
@@ -3011,16 +3250,19 @@
       <c r="L41">
         <v>66</v>
       </c>
-      <c r="M41" t="b">
-        <v>1</v>
-      </c>
-      <c r="N41">
-        <v>93.33333333333333</v>
+      <c r="M41">
+        <v>15</v>
+      </c>
+      <c r="N41" t="b">
+        <v>1</v>
       </c>
       <c r="O41">
         <v>93.33333333333333</v>
       </c>
       <c r="P41">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q41">
         <v>92.95774647887323</v>
       </c>
     </row>
@@ -3071,16 +3313,19 @@
       <c r="L42">
         <v>55</v>
       </c>
-      <c r="M42" t="b">
-        <v>1</v>
-      </c>
-      <c r="N42">
-        <v>86.66666666666667</v>
+      <c r="M42">
+        <v>15</v>
+      </c>
+      <c r="N42" t="b">
+        <v>1</v>
       </c>
       <c r="O42">
         <v>86.66666666666667</v>
       </c>
       <c r="P42">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q42">
         <v>84.61538461538461</v>
       </c>
     </row>
@@ -3131,11 +3376,11 @@
       <c r="L43">
         <v>81</v>
       </c>
-      <c r="M43" t="b">
-        <v>1</v>
-      </c>
-      <c r="N43">
-        <v>100</v>
+      <c r="M43">
+        <v>15</v>
+      </c>
+      <c r="N43" t="b">
+        <v>1</v>
       </c>
       <c r="O43">
         <v>100</v>
@@ -3143,6 +3388,9 @@
       <c r="P43">
         <v>100</v>
       </c>
+      <c r="Q43">
+        <v>100</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3191,16 +3439,19 @@
       <c r="L44">
         <v>61</v>
       </c>
-      <c r="M44" t="b">
-        <v>1</v>
-      </c>
-      <c r="N44">
-        <v>86.66666666666667</v>
+      <c r="M44">
+        <v>15</v>
+      </c>
+      <c r="N44" t="b">
+        <v>1</v>
       </c>
       <c r="O44">
         <v>86.66666666666667</v>
       </c>
       <c r="P44">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q44">
         <v>85.91549295774648</v>
       </c>
     </row>
@@ -3251,16 +3502,19 @@
       <c r="L45">
         <v>72</v>
       </c>
-      <c r="M45" t="b">
-        <v>1</v>
-      </c>
-      <c r="N45">
-        <v>93.33333333333333</v>
+      <c r="M45">
+        <v>15</v>
+      </c>
+      <c r="N45" t="b">
+        <v>1</v>
       </c>
       <c r="O45">
         <v>93.33333333333333</v>
       </c>
       <c r="P45">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q45">
         <v>96</v>
       </c>
     </row>
@@ -3311,16 +3565,19 @@
       <c r="L46">
         <v>64</v>
       </c>
-      <c r="M46" t="b">
-        <v>1</v>
-      </c>
-      <c r="N46">
-        <v>80</v>
+      <c r="M46">
+        <v>15</v>
+      </c>
+      <c r="N46" t="b">
+        <v>1</v>
       </c>
       <c r="O46">
         <v>80</v>
       </c>
       <c r="P46">
+        <v>80</v>
+      </c>
+      <c r="Q46">
         <v>83.11688311688312</v>
       </c>
     </row>
@@ -3371,16 +3628,19 @@
       <c r="L47">
         <v>60</v>
       </c>
-      <c r="M47" t="b">
-        <v>1</v>
-      </c>
-      <c r="N47">
-        <v>66.66666666666666</v>
+      <c r="M47">
+        <v>15</v>
+      </c>
+      <c r="N47" t="b">
+        <v>1</v>
       </c>
       <c r="O47">
         <v>66.66666666666666</v>
       </c>
       <c r="P47">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="Q47">
         <v>74.07407407407408</v>
       </c>
     </row>
@@ -3431,11 +3691,11 @@
       <c r="L48">
         <v>55</v>
       </c>
-      <c r="M48" t="b">
-        <v>1</v>
-      </c>
-      <c r="N48">
-        <v>73.33333333333333</v>
+      <c r="M48">
+        <v>15</v>
+      </c>
+      <c r="N48" t="b">
+        <v>1</v>
       </c>
       <c r="O48">
         <v>73.33333333333333</v>
@@ -3443,6 +3703,9 @@
       <c r="P48">
         <v>73.33333333333333</v>
       </c>
+      <c r="Q48">
+        <v>73.33333333333333</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3491,16 +3754,19 @@
       <c r="L49">
         <v>57</v>
       </c>
-      <c r="M49" t="b">
-        <v>1</v>
-      </c>
-      <c r="N49">
-        <v>73.33333333333333</v>
+      <c r="M49">
+        <v>15</v>
+      </c>
+      <c r="N49" t="b">
+        <v>1</v>
       </c>
       <c r="O49">
         <v>73.33333333333333</v>
       </c>
       <c r="P49">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q49">
         <v>78.08219178082192</v>
       </c>
     </row>
@@ -3551,11 +3817,11 @@
       <c r="L50">
         <v>42</v>
       </c>
-      <c r="M50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N50">
-        <v>66.66666666666666</v>
+      <c r="M50">
+        <v>15</v>
+      </c>
+      <c r="N50" t="b">
+        <v>1</v>
       </c>
       <c r="O50">
         <v>66.66666666666666</v>
@@ -3563,6 +3829,9 @@
       <c r="P50">
         <v>66.66666666666666</v>
       </c>
+      <c r="Q50">
+        <v>66.66666666666666</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3611,16 +3880,19 @@
       <c r="L51">
         <v>61</v>
       </c>
-      <c r="M51" t="b">
-        <v>1</v>
-      </c>
-      <c r="N51">
-        <v>73.33333333333333</v>
+      <c r="M51">
+        <v>15</v>
+      </c>
+      <c r="N51" t="b">
+        <v>1</v>
       </c>
       <c r="O51">
         <v>73.33333333333333</v>
       </c>
       <c r="P51">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q51">
         <v>77.21518987341773</v>
       </c>
     </row>
@@ -3671,11 +3943,11 @@
       <c r="L52">
         <v>60</v>
       </c>
-      <c r="M52" t="b">
-        <v>1</v>
-      </c>
-      <c r="N52">
-        <v>80</v>
+      <c r="M52">
+        <v>15</v>
+      </c>
+      <c r="N52" t="b">
+        <v>1</v>
       </c>
       <c r="O52">
         <v>80</v>
@@ -3683,6 +3955,9 @@
       <c r="P52">
         <v>80</v>
       </c>
+      <c r="Q52">
+        <v>80</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3731,11 +4006,11 @@
       <c r="L53">
         <v>45</v>
       </c>
-      <c r="M53" t="b">
-        <v>1</v>
-      </c>
-      <c r="N53">
-        <v>60</v>
+      <c r="M53">
+        <v>15</v>
+      </c>
+      <c r="N53" t="b">
+        <v>1</v>
       </c>
       <c r="O53">
         <v>60</v>
@@ -3743,6 +4018,9 @@
       <c r="P53">
         <v>60</v>
       </c>
+      <c r="Q53">
+        <v>60</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3791,16 +4069,19 @@
       <c r="L54">
         <v>66</v>
       </c>
-      <c r="M54" t="b">
-        <v>1</v>
-      </c>
-      <c r="N54">
-        <v>80</v>
+      <c r="M54">
+        <v>15</v>
+      </c>
+      <c r="N54" t="b">
+        <v>1</v>
       </c>
       <c r="O54">
         <v>80</v>
       </c>
       <c r="P54">
+        <v>80</v>
+      </c>
+      <c r="Q54">
         <v>88</v>
       </c>
     </row>
@@ -3851,16 +4132,19 @@
       <c r="L55">
         <v>58</v>
       </c>
-      <c r="M55" t="b">
-        <v>1</v>
-      </c>
-      <c r="N55">
-        <v>80</v>
+      <c r="M55">
+        <v>15</v>
+      </c>
+      <c r="N55" t="b">
+        <v>1</v>
       </c>
       <c r="O55">
         <v>80</v>
       </c>
       <c r="P55">
+        <v>80</v>
+      </c>
+      <c r="Q55">
         <v>79.45205479452055</v>
       </c>
     </row>
@@ -3911,16 +4195,19 @@
       <c r="L56">
         <v>57</v>
       </c>
-      <c r="M56" t="b">
-        <v>1</v>
-      </c>
-      <c r="N56">
-        <v>86.66666666666667</v>
+      <c r="M56">
+        <v>15</v>
+      </c>
+      <c r="N56" t="b">
+        <v>1</v>
       </c>
       <c r="O56">
         <v>86.66666666666667</v>
       </c>
       <c r="P56">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q56">
         <v>85.07462686567165</v>
       </c>
     </row>
@@ -3971,16 +4258,19 @@
       <c r="L57">
         <v>60</v>
       </c>
-      <c r="M57" t="b">
-        <v>1</v>
-      </c>
-      <c r="N57">
-        <v>66.66666666666666</v>
+      <c r="M57">
+        <v>15</v>
+      </c>
+      <c r="N57" t="b">
+        <v>1</v>
       </c>
       <c r="O57">
         <v>66.66666666666666</v>
       </c>
       <c r="P57">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="Q57">
         <v>74.07407407407408</v>
       </c>
     </row>
@@ -4031,16 +4321,19 @@
       <c r="L58">
         <v>66</v>
       </c>
-      <c r="M58" t="b">
-        <v>1</v>
-      </c>
-      <c r="N58">
-        <v>80</v>
+      <c r="M58">
+        <v>15</v>
+      </c>
+      <c r="N58" t="b">
+        <v>1</v>
       </c>
       <c r="O58">
         <v>80</v>
       </c>
       <c r="P58">
+        <v>80</v>
+      </c>
+      <c r="Q58">
         <v>83.54430379746836</v>
       </c>
     </row>
@@ -4091,16 +4384,19 @@
       <c r="L59">
         <v>70</v>
       </c>
-      <c r="M59" t="b">
-        <v>1</v>
-      </c>
-      <c r="N59">
-        <v>93.33333333333333</v>
+      <c r="M59">
+        <v>15</v>
+      </c>
+      <c r="N59" t="b">
+        <v>1</v>
       </c>
       <c r="O59">
         <v>93.33333333333333</v>
       </c>
       <c r="P59">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q59">
         <v>90.90909090909091</v>
       </c>
     </row>
@@ -4151,16 +4447,19 @@
       <c r="L60">
         <v>61</v>
       </c>
-      <c r="M60" t="b">
-        <v>1</v>
-      </c>
-      <c r="N60">
-        <v>73.33333333333333</v>
+      <c r="M60">
+        <v>15</v>
+      </c>
+      <c r="N60" t="b">
+        <v>1</v>
       </c>
       <c r="O60">
         <v>73.33333333333333</v>
       </c>
       <c r="P60">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q60">
         <v>77.21518987341773</v>
       </c>
     </row>
@@ -4211,16 +4510,19 @@
       <c r="L61">
         <v>72</v>
       </c>
-      <c r="M61" t="b">
-        <v>1</v>
-      </c>
-      <c r="N61">
-        <v>93.33333333333333</v>
+      <c r="M61">
+        <v>15</v>
+      </c>
+      <c r="N61" t="b">
+        <v>1</v>
       </c>
       <c r="O61">
         <v>93.33333333333333</v>
       </c>
       <c r="P61">
+        <v>93.33333333333333</v>
+      </c>
+      <c r="Q61">
         <v>91.13924050632912</v>
       </c>
     </row>
@@ -4271,16 +4573,19 @@
       <c r="L62">
         <v>59</v>
       </c>
-      <c r="M62" t="b">
-        <v>1</v>
-      </c>
-      <c r="N62">
-        <v>73.33333333333333</v>
+      <c r="M62">
+        <v>15</v>
+      </c>
+      <c r="N62" t="b">
+        <v>1</v>
       </c>
       <c r="O62">
         <v>73.33333333333333</v>
       </c>
       <c r="P62">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q62">
         <v>76.62337662337663</v>
       </c>
     </row>
@@ -4331,16 +4636,19 @@
       <c r="L63">
         <v>34</v>
       </c>
-      <c r="M63" t="b">
-        <v>1</v>
-      </c>
-      <c r="N63">
-        <v>40</v>
+      <c r="M63">
+        <v>15</v>
+      </c>
+      <c r="N63" t="b">
+        <v>1</v>
       </c>
       <c r="O63">
         <v>40</v>
       </c>
       <c r="P63">
+        <v>40</v>
+      </c>
+      <c r="Q63">
         <v>50.74626865671642</v>
       </c>
     </row>
@@ -4391,11 +4699,11 @@
       <c r="L64">
         <v>68</v>
       </c>
-      <c r="M64" t="b">
-        <v>1</v>
-      </c>
-      <c r="N64">
-        <v>80</v>
+      <c r="M64">
+        <v>15</v>
+      </c>
+      <c r="N64" t="b">
+        <v>1</v>
       </c>
       <c r="O64">
         <v>80</v>
@@ -4403,6 +4711,9 @@
       <c r="P64">
         <v>80</v>
       </c>
+      <c r="Q64">
+        <v>80</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4451,16 +4762,19 @@
       <c r="L65">
         <v>77</v>
       </c>
-      <c r="M65" t="b">
-        <v>1</v>
-      </c>
-      <c r="N65">
-        <v>86.66666666666667</v>
+      <c r="M65">
+        <v>15</v>
+      </c>
+      <c r="N65" t="b">
+        <v>1</v>
       </c>
       <c r="O65">
         <v>86.66666666666667</v>
       </c>
       <c r="P65">
+        <v>86.66666666666667</v>
+      </c>
+      <c r="Q65">
         <v>92.77108433734939</v>
       </c>
     </row>
@@ -4511,16 +4825,19 @@
       <c r="L66">
         <v>43</v>
       </c>
-      <c r="M66" t="b">
-        <v>1</v>
-      </c>
-      <c r="N66">
-        <v>73.33333333333333</v>
+      <c r="M66">
+        <v>15</v>
+      </c>
+      <c r="N66" t="b">
+        <v>1</v>
       </c>
       <c r="O66">
         <v>73.33333333333333</v>
       </c>
       <c r="P66">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q66">
         <v>72.88135593220339</v>
       </c>
     </row>
@@ -4571,16 +4888,19 @@
       <c r="L67">
         <v>59</v>
       </c>
-      <c r="M67" t="b">
-        <v>1</v>
-      </c>
-      <c r="N67">
-        <v>73.33333333333333</v>
+      <c r="M67">
+        <v>15</v>
+      </c>
+      <c r="N67" t="b">
+        <v>1</v>
       </c>
       <c r="O67">
         <v>73.33333333333333</v>
       </c>
       <c r="P67">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="Q67">
         <v>74.68354430379746</v>
       </c>
     </row>
@@ -4631,16 +4951,19 @@
       <c r="L68">
         <v>42</v>
       </c>
-      <c r="M68" t="b">
-        <v>1</v>
-      </c>
-      <c r="N68">
-        <v>53.33333333333334</v>
+      <c r="M68">
+        <v>15</v>
+      </c>
+      <c r="N68" t="b">
+        <v>1</v>
       </c>
       <c r="O68">
         <v>53.33333333333334</v>
       </c>
       <c r="P68">
+        <v>53.33333333333334</v>
+      </c>
+      <c r="Q68">
         <v>54.54545454545454</v>
       </c>
     </row>
@@ -4779,7 +5102,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -4810,6 +5133,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>unanswered_answers</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>accuracy_percent</t>
         </is>
       </c>
@@ -4833,6 +5161,9 @@
         <v>80</v>
       </c>
       <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
         <v>79.64376590330788</v>
       </c>
     </row>
@@ -4855,6 +5186,9 @@
         <v>6</v>
       </c>
       <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
         <v>78.57142857142857</v>
       </c>
     </row>
@@ -4877,6 +5211,9 @@
         <v>15</v>
       </c>
       <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
         <v>85.57692307692307</v>
       </c>
     </row>
@@ -4899,6 +5236,9 @@
         <v>50</v>
       </c>
       <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
         <v>85.71428571428571</v>
       </c>
     </row>
@@ -4921,6 +5261,9 @@
         <v>17</v>
       </c>
       <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
         <v>63.82978723404256</v>
       </c>
     </row>
@@ -4943,6 +5286,9 @@
         <v>13</v>
       </c>
       <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
         <v>84.33734939759037</v>
       </c>
     </row>
@@ -5097,7 +5443,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -5118,6 +5464,16 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>correct_answers</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>wrong_answers</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>accuracy_percent</t>
         </is>
       </c>
@@ -5133,6 +5489,12 @@
         <v>39</v>
       </c>
       <c r="D2">
+        <v>31</v>
+      </c>
+      <c r="E2">
+        <v>8</v>
+      </c>
+      <c r="F2">
         <v>79.48717948717949</v>
       </c>
     </row>
@@ -5147,6 +5509,12 @@
         <v>112</v>
       </c>
       <c r="D3">
+        <v>80</v>
+      </c>
+      <c r="E3">
+        <v>32</v>
+      </c>
+      <c r="F3">
         <v>71.42857142857143</v>
       </c>
     </row>
@@ -5161,6 +5529,12 @@
         <v>178</v>
       </c>
       <c r="D4">
+        <v>141</v>
+      </c>
+      <c r="E4">
+        <v>37</v>
+      </c>
+      <c r="F4">
         <v>79.21348314606742</v>
       </c>
     </row>
@@ -5175,6 +5549,12 @@
         <v>196</v>
       </c>
       <c r="D5">
+        <v>172</v>
+      </c>
+      <c r="E5">
+        <v>24</v>
+      </c>
+      <c r="F5">
         <v>87.75510204081633</v>
       </c>
     </row>
@@ -5189,6 +5569,12 @@
         <v>48</v>
       </c>
       <c r="D6">
+        <v>40</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+      <c r="F6">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -5203,6 +5589,12 @@
         <v>91</v>
       </c>
       <c r="D7">
+        <v>68</v>
+      </c>
+      <c r="E7">
+        <v>23</v>
+      </c>
+      <c r="F7">
         <v>74.72527472527473</v>
       </c>
     </row>
@@ -5217,6 +5609,12 @@
         <v>174</v>
       </c>
       <c r="D8">
+        <v>143</v>
+      </c>
+      <c r="E8">
+        <v>31</v>
+      </c>
+      <c r="F8">
         <v>82.18390804597702</v>
       </c>
     </row>
@@ -5231,6 +5629,12 @@
         <v>167</v>
       </c>
       <c r="D9">
+        <v>149</v>
+      </c>
+      <c r="E9">
+        <v>18</v>
+      </c>
+      <c r="F9">
         <v>89.22155688622755</v>
       </c>
     </row>
@@ -5241,7 +5645,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -5277,10 +5681,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>unanswered_count</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>accuracy_percent</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>mean_weight</t>
         </is>
@@ -5306,9 +5715,12 @@
         <v>5</v>
       </c>
       <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
         <v>85.71428571428571</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>4.828571428571428</v>
       </c>
     </row>
@@ -5332,9 +5744,12 @@
         <v>4</v>
       </c>
       <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
         <v>88.57142857142857</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>4.828571428571428</v>
       </c>
     </row>
@@ -5358,9 +5773,12 @@
         <v>9</v>
       </c>
       <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
         <v>74.28571428571429</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>4.828571428571428</v>
       </c>
     </row>
@@ -5384,9 +5802,12 @@
         <v>2</v>
       </c>
       <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
         <v>94.28571428571428</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>5.228571428571429</v>
       </c>
     </row>
@@ -5410,9 +5831,12 @@
         <v>9</v>
       </c>
       <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>74.28571428571429</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>5.4</v>
       </c>
     </row>
@@ -5436,9 +5860,12 @@
         <v>7</v>
       </c>
       <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
         <v>80</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>5.342857142857143</v>
       </c>
     </row>
@@ -5462,9 +5889,12 @@
         <v>2</v>
       </c>
       <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
         <v>94.28571428571428</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>5.514285714285714</v>
       </c>
     </row>
@@ -5488,9 +5918,12 @@
         <v>12</v>
       </c>
       <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
         <v>65.71428571428571</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>5</v>
       </c>
     </row>
@@ -5514,9 +5947,12 @@
         <v>6</v>
       </c>
       <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
         <v>82.85714285714286</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>4.428571428571429</v>
       </c>
     </row>
@@ -5540,9 +5976,12 @@
         <v>7</v>
       </c>
       <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
         <v>80</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>4.542857142857143</v>
       </c>
     </row>
@@ -5566,9 +6005,12 @@
         <v>7</v>
       </c>
       <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
         <v>80</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>5.057142857142857</v>
       </c>
     </row>
@@ -5592,9 +6034,12 @@
         <v>11</v>
       </c>
       <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
         <v>68.57142857142857</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>5.171428571428572</v>
       </c>
     </row>
@@ -5618,9 +6063,12 @@
         <v>8</v>
       </c>
       <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
         <v>77.14285714285715</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>5.228571428571429</v>
       </c>
     </row>
@@ -5644,9 +6092,12 @@
         <v>4</v>
       </c>
       <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
         <v>88.57142857142857</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>5.171428571428572</v>
       </c>
     </row>
@@ -5670,9 +6121,12 @@
         <v>8</v>
       </c>
       <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
         <v>77.14285714285715</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>4.771428571428571</v>
       </c>
     </row>
@@ -5696,9 +6150,12 @@
         <v>4</v>
       </c>
       <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
         <v>87.5</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>5.375</v>
       </c>
     </row>
@@ -5722,9 +6179,12 @@
         <v>7</v>
       </c>
       <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
         <v>78.125</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>5.125</v>
       </c>
     </row>
@@ -5748,9 +6208,12 @@
         <v>5</v>
       </c>
       <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
         <v>84.375</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>4.75</v>
       </c>
     </row>
@@ -5774,9 +6237,12 @@
         <v>3</v>
       </c>
       <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
         <v>90.625</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>5.25</v>
       </c>
     </row>
@@ -5800,9 +6266,12 @@
         <v>7</v>
       </c>
       <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
         <v>78.125</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>4.6875</v>
       </c>
     </row>
@@ -5826,9 +6295,12 @@
         <v>6</v>
       </c>
       <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
         <v>81.25</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>4.8125</v>
       </c>
     </row>
@@ -5852,9 +6324,12 @@
         <v>7</v>
       </c>
       <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
         <v>78.125</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>4.375</v>
       </c>
     </row>
@@ -5878,9 +6353,12 @@
         <v>4</v>
       </c>
       <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
         <v>87.5</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>5.5</v>
       </c>
     </row>
@@ -5904,9 +6382,12 @@
         <v>6</v>
       </c>
       <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
         <v>81.25</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>4.5</v>
       </c>
     </row>
@@ -5930,9 +6411,12 @@
         <v>7</v>
       </c>
       <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
         <v>78.125</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>5.125</v>
       </c>
     </row>
@@ -5956,9 +6440,12 @@
         <v>2</v>
       </c>
       <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
         <v>93.75</v>
       </c>
-      <c r="H27">
+      <c r="I27">
         <v>4.8125</v>
       </c>
     </row>
@@ -5982,9 +6469,12 @@
         <v>8</v>
       </c>
       <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
         <v>75</v>
       </c>
-      <c r="H28">
+      <c r="I28">
         <v>5.0625</v>
       </c>
     </row>
@@ -6008,9 +6498,12 @@
         <v>8</v>
       </c>
       <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
         <v>75</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>5.125</v>
       </c>
     </row>
@@ -6034,9 +6527,12 @@
         <v>3</v>
       </c>
       <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
         <v>90.625</v>
       </c>
-      <c r="H30">
+      <c r="I30">
         <v>4.1875</v>
       </c>
     </row>
@@ -6060,9 +6556,12 @@
         <v>3</v>
       </c>
       <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
         <v>90.625</v>
       </c>
-      <c r="H31">
+      <c r="I31">
         <v>5.0625</v>
       </c>
     </row>
@@ -6379,4 +6878,721 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>total_responses</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mean_score</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>sd_score</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>median_score</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>negative_percent</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>neutral_percent</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>positive_percent</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>item_01</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>34</v>
+      </c>
+      <c r="C2">
+        <v>4.705882352941177</v>
+      </c>
+      <c r="D2">
+        <v>0.4624972900628804</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>100</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>item_02</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>34</v>
+      </c>
+      <c r="C3">
+        <v>4.676470588235294</v>
+      </c>
+      <c r="D3">
+        <v>0.5348796656113336</v>
+      </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="H3">
+        <v>97.05882352941177</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>item_03</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>34</v>
+      </c>
+      <c r="C4">
+        <v>4.558823529411764</v>
+      </c>
+      <c r="D4">
+        <v>0.6125543375075285</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>5.88235294117647</v>
+      </c>
+      <c r="H4">
+        <v>94.11764705882352</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>item_04</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>34</v>
+      </c>
+      <c r="C5">
+        <v>4.588235294117647</v>
+      </c>
+      <c r="D5">
+        <v>0.6089059766610498</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>5.88235294117647</v>
+      </c>
+      <c r="H5">
+        <v>94.11764705882352</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>item_05</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>34</v>
+      </c>
+      <c r="C6">
+        <v>4.558823529411764</v>
+      </c>
+      <c r="D6">
+        <v>0.6601733689004337</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>8.823529411764707</v>
+      </c>
+      <c r="H6">
+        <v>91.17647058823529</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>item_06</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>34</v>
+      </c>
+      <c r="C7">
+        <v>4.823529411764706</v>
+      </c>
+      <c r="D7">
+        <v>0.3869529949759475</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>100</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>item_07</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>34</v>
+      </c>
+      <c r="C8">
+        <v>4.617647058823529</v>
+      </c>
+      <c r="D8">
+        <v>0.5512908203729233</v>
+      </c>
+      <c r="E8">
+        <v>5</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="H8">
+        <v>97.05882352941177</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>item_08</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>34</v>
+      </c>
+      <c r="C9">
+        <v>4.529411764705882</v>
+      </c>
+      <c r="D9">
+        <v>0.5632854982907604</v>
+      </c>
+      <c r="E9">
+        <v>5</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="H9">
+        <v>97.05882352941177</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>item_09</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>34</v>
+      </c>
+      <c r="C10">
+        <v>4.647058823529412</v>
+      </c>
+      <c r="D10">
+        <v>0.6911717297975236</v>
+      </c>
+      <c r="E10">
+        <v>5</v>
+      </c>
+      <c r="F10">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="G10">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="H10">
+        <v>94.11764705882352</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>item_10</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>34</v>
+      </c>
+      <c r="C11">
+        <v>4.617647058823529</v>
+      </c>
+      <c r="D11">
+        <v>0.6037612352855318</v>
+      </c>
+      <c r="E11">
+        <v>5</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>5.88235294117647</v>
+      </c>
+      <c r="H11">
+        <v>94.11764705882352</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>item_11</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>34</v>
+      </c>
+      <c r="C12">
+        <v>4.647058823529412</v>
+      </c>
+      <c r="D12">
+        <v>0.5970814340265321</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>5.88235294117647</v>
+      </c>
+      <c r="H12">
+        <v>94.11764705882352</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>item_12</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>34</v>
+      </c>
+      <c r="C13">
+        <v>4.352941176470588</v>
+      </c>
+      <c r="D13">
+        <v>0.8835998319950068</v>
+      </c>
+      <c r="E13">
+        <v>5</v>
+      </c>
+      <c r="F13">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="G13">
+        <v>17.64705882352941</v>
+      </c>
+      <c r="H13">
+        <v>79.41176470588235</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>item_13</t>
+        </is>
+      </c>
+      <c r="B14">
+        <v>34</v>
+      </c>
+      <c r="C14">
+        <v>4.470588235294118</v>
+      </c>
+      <c r="D14">
+        <v>0.8251829592405758</v>
+      </c>
+      <c r="E14">
+        <v>5</v>
+      </c>
+      <c r="F14">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="G14">
+        <v>11.76470588235294</v>
+      </c>
+      <c r="H14">
+        <v>85.29411764705883</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>item_14</t>
+        </is>
+      </c>
+      <c r="B15">
+        <v>34</v>
+      </c>
+      <c r="C15">
+        <v>4.264705882352941</v>
+      </c>
+      <c r="D15">
+        <v>1.136417111041267</v>
+      </c>
+      <c r="E15">
+        <v>5</v>
+      </c>
+      <c r="F15">
+        <v>11.76470588235294</v>
+      </c>
+      <c r="G15">
+        <v>8.823529411764707</v>
+      </c>
+      <c r="H15">
+        <v>79.41176470588235</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>item_15</t>
+        </is>
+      </c>
+      <c r="B16">
+        <v>34</v>
+      </c>
+      <c r="C16">
+        <v>4.588235294117647</v>
+      </c>
+      <c r="D16">
+        <v>0.656789577429185</v>
+      </c>
+      <c r="E16">
+        <v>5</v>
+      </c>
+      <c r="F16">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>97.05882352941177</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>item_16</t>
+        </is>
+      </c>
+      <c r="B17">
+        <v>34</v>
+      </c>
+      <c r="C17">
+        <v>4.588235294117647</v>
+      </c>
+      <c r="D17">
+        <v>0.6567895774291852</v>
+      </c>
+      <c r="E17">
+        <v>5</v>
+      </c>
+      <c r="F17">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>97.05882352941177</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>item_17</t>
+        </is>
+      </c>
+      <c r="B18">
+        <v>34</v>
+      </c>
+      <c r="C18">
+        <v>4.588235294117647</v>
+      </c>
+      <c r="D18">
+        <v>0.7014118687516404</v>
+      </c>
+      <c r="E18">
+        <v>5</v>
+      </c>
+      <c r="F18">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="G18">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="H18">
+        <v>94.11764705882352</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>item_18</t>
+        </is>
+      </c>
+      <c r="B19">
+        <v>34</v>
+      </c>
+      <c r="C19">
+        <v>4.676470588235294</v>
+      </c>
+      <c r="D19">
+        <v>0.5348796656113336</v>
+      </c>
+      <c r="E19">
+        <v>5</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="H19">
+        <v>97.05882352941177</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>item_19</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>34</v>
+      </c>
+      <c r="C20">
+        <v>4.705882352941177</v>
+      </c>
+      <c r="D20">
+        <v>0.6755205294731985</v>
+      </c>
+      <c r="E20">
+        <v>5</v>
+      </c>
+      <c r="F20">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="G20">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="H20">
+        <v>94.11764705882352</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>item_20</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>34</v>
+      </c>
+      <c r="C21">
+        <v>4.529411764705882</v>
+      </c>
+      <c r="D21">
+        <v>0.7064762801416987</v>
+      </c>
+      <c r="E21">
+        <v>5</v>
+      </c>
+      <c r="F21">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="G21">
+        <v>2.941176470588235</v>
+      </c>
+      <c r="H21">
+        <v>94.11764705882352</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Sangat Tinggi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>